<commit_message>
feat: add improvements for whatsapp template variables
</commit_message>
<xml_diff>
--- a/public/bulk-insert-clients.xlsx
+++ b/public/bulk-insert-clients.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJETOS\recompracrm\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D7844052-0164-47B0-8A27-312EDF3D79F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{889DFB69-6D2C-40DB-9224-0A9698A1F247}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6795" yWindow="3090" windowWidth="21600" windowHeight="11295" xr2:uid="{1E8F4C92-23D7-4F89-9802-D0DC771B31B9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1E8F4C92-23D7-4F89-9802-D0DC771B31B9}"/>
   </bookViews>
   <sheets>
-    <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
+    <sheet name="CLIENTES" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -70,7 +70,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -90,6 +90,15 @@
       <u/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -121,7 +130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -130,6 +139,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -454,7 +466,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" s="2" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">

</xml_diff>